<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.001-02 Sarah dit stop, puis encore
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.001-02.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.001-02.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La ronde trop vite</t>
+          <t>Sarah dit stop, puis encore</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>maison puis jardin</t>
+          <t>maison, rideau, fenêtre, linge, soleil, bois, jardin, herbe, porte, fleurs, panier</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Victorino, Aniss, papa</t>
+          <t>Sarah, Aniss, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorino tourne avec Aniss. C'est trop vite. Il dit stop, s'éloigne, rejoint papa. Au jardin, la ronde recommence. Il dit stop encore.</t>
+          <t>Le linge tiède bouge devant le jardin. Près du tissu, un éclat de rideau brille. Sarah veut la ronde maintenant. Aniss tourne trop. Poitrine coincée, sourire parti, papa accroupi. Stop, recule. Merci vécu. Deuxième ruse : trop vite au jardin. Elle dit stop. Un éclat de rideau tient sur le tissu.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une bande de soleil rampe sur le plancher. Le bois est tiède sous les pieds nus. La maison sent le pain chaud. Un moulin en papier tourne à la fenêtre. Il fait un petit bruit doux. Papa range des livres près du canapé. Les livres tapent tout bas. J'aime ce petit bruit, Victorino. Tu as entendu le moulin ? Oui, papa. Il tourne. Le tapis beige est épais. En ce moment, Victorino joue avec Aniss. Ils se tiennent par les mains. Ils tournent au milieu du salon. Le tapis tourne autour d'eux. Plus vite, Aniss ! Aniss tourne plus vite. Trop vite. Victorino est gêné. Aniss le tourne trop fort. Sa poitrine est coincée. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Victorino recule d'un pas. Il peut s'éloigner. Il s'éloigne vers le canapé. Papa est l'adulte près du canapé. Papa, c'était trop. Tu as dit stop. Bravo, Victorino. Tu t'es éloigné. Tu es venu vers moi. Tu veux t'asseoir un peu ? Oui, papa. Victorino pose sa main dans la main de papa. Il souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Plus tard, la porte du jardin cliquette. L'herbe sent le thym. Un seau jaune attend près des fleurs. Aniss veut une ronde. Il prend la main de Victorino. La ronde commence. Trop près. Trop vite encore. Victorino sent encore sa poitrine coincée. Il se souvient. Stop. Il s'éloigne. Il va vers papa, l'adulte. Papa, c'est trop encore. Tu as repris le geste. Bravo. Tu as dit stop au jardin aussi. Tu t'es éloigné. Tu es venu vers un adulte. Vers moi. Victorino reste près de papa. Ses épaules descendent. Aniss joue avec le seau jaune. Le seau tapote l'herbe.</t>
+          <t>Le linge tiède bouge devant le jardin. Ça sent le pain et le soleil. Ça sent le pain, papa. Tu le sens, le linge, Sarah ? Oui, papa. Un rai passe à travers le tissu. Le tissu fait un bruit court. Il claque, maman. Le tissu tient près du bois ? Oui, maman. Près du tissu, un éclat de rideau brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. La fenêtre tient un bout de jardin pâle. Il est clair, papa. Le jardin, là-bas ? Oui, là-bas. Aniss tend les mains vers Sarah. On tourne, Sarah ! On tourne, maintenant ! La ronde, avec Aniss ? Oui. Tout de suite. En ce moment, Sarah se penche vers lui. Leurs mains se tiennent. Plus vite ! Aniss tourne trop vite. Le tissu claque un peu. Sarah veut la ronde, elle aussi. Plus vite ! Le tourbillon serre trop. Sa poitrine est coincée. Le sourire de Sarah disparaît. Ses épaules montent. Oh. Tu vois Aniss, Sarah ? Oui, papa. Tes épaules sont hautes, Sarah ? Un peu, maman. L'éclat de rideau tremble, puis tient. Sarah serre les mains trop fort. C'est trop, papa. Papa s'accroupit à la même hauteur. Sarah regarde papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une bande de soleil rampe sur le plancher. Le bois est tiède sous les pieds nus. La maison sent le pain chaud. Un moulin en papier tourne à la fenêtre. Il fait un petit bruit doux. Papa range des livres près du canapé. Les livres tapent tout bas. J'aime ce petit bruit, Victorino. Tu as entendu le moulin ? Oui, papa. Il tourne. Le tapis beige est épais. En ce moment, Victorino joue avec Aniss. Ils se tiennent par les mains. Ils tournent au milieu du salon. Le tapis tourne autour d'eux. Plus vite, Aniss ! Aniss tourne plus vite. Trop vite. Victorino est gêné. Aniss le tourne trop fort. Sa poitrine est coincée. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Victorino recule d'un pas. Il peut s'éloigner. Il s'éloigne vers le canapé. Papa est l'adulte près du canapé. Papa, c'était trop. Tu as dit stop. Bravo, Victorino. Tu t'es éloigné. Tu es venu vers moi. Tu veux t'asseoir un peu ? Oui, papa. Victorino pose sa main dans la main de papa. Il souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Plus tard, la porte du jardin cliquette. L'herbe sent le thym. Un seau jaune attend près des fleurs. Aniss veut une ronde. Il prend la main de Victorino. La ronde commence. Trop près. Trop vite encore. Victorino sent encore sa poitrine coincée. Il se souvient. Stop. Il s'éloigne. Il va vers papa, l'adulte. Papa, c'est trop encore. Tu as repris le geste. Bravo. Tu as dit stop au jardin aussi. Tu t'es éloigné. Tu es venu vers un adulte. Vers moi. Victorino reste près de papa. Ses épaules descendent. Aniss joue avec le seau jaune. Le seau tapote l'herbe.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le linge tiède bouge devant le jardin. Ça sent le pain et le soleil. Ça sent le pain, papa. Tu le sens, le linge, Sarah ? Oui, papa. Un rai passe à travers le tissu. Le tissu fait un bruit court. Il claque, maman. Le tissu tient près du bois ? Oui, maman. Près du tissu, un &lt;emphasis level="moderate"&gt;éclat de rideau&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. La fenêtre tient un bout de jardin pâle. Il est clair, papa. Le jardin, là-bas ? Oui, là-bas. Aniss tend les mains vers Sarah. On tourne, Sarah ! On tourne, maintenant ! La ronde, avec Aniss ? Oui. Tout de suite. En ce moment, Sarah se penche vers lui. Leurs mains se tiennent. Plus vite ! Aniss tourne trop vite. Le tissu claque un peu. Sarah veut la ronde, elle aussi. Plus vite ! Le tourbillon serre trop. Sa poitrine est coincée. Le sourire de Sarah disparaît. Ses épaules montent. Oh. Tu vois Aniss, Sarah ? Oui, papa. Tes épaules sont hautes, Sarah ? Un peu, maman. L'éclat de rideau tremble, puis tient. Sarah serre les mains trop fort. C'est trop, papa. Papa s'accroupit à la même hauteur. Sarah regarde papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Sara joue dans le salon avec papa. Un camarade la tourne trop vite. Sara sent sa poitrine coincée. Elle dit : je n'aime pas. C'est trop. Sara dit : &lt;emphasis&gt;stop&lt;/emphasis&gt;. Elle recule d'un pas. Elle peut s'éloigner. Elle s'éloigne vers le canapé. Papa est l'adulte près du canapé. Sara va vers papa. Elle dit : c'était trop. Papa l'écoute. Sara pose sa main dans la main de papa. Elle souffle. Plus tard, ils vont au jardin. Les enfants font une ronde. On la serre trop près. Sara sent encore la poitrine coincée. Elle se souvient. Elle dit : stop. Elle s'éloigne. Elle va vers papa, l'adulte. Papa dit : tu as repris le geste. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Même leçon, autre lieu. Sara reste près de papa. Ses épaules descendent. [pause]</t>
+          <t>Le linge tiède bouge devant le jardin. Ça sent le pain et le soleil. Ça sent le pain, papa. Tu le sens, le linge, Sarah ? Oui, papa. Un rai passe à travers le tissu. Le tissu fait un bruit court. Il claque, maman. Le tissu tient près du bois ? Oui, maman. Près du tissu, un &lt;emphasis&gt;éclat de rideau&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. La fenêtre tient un bout de jardin pâle. Il est clair, papa. Le jardin, là-bas ? Oui, là-bas. Aniss tend les mains vers Sarah. On tourne, Sarah ! On tourne, maintenant ! La ronde, avec Aniss ? Oui. Tout de suite. En ce moment, Sarah se penche vers lui. Leurs mains se tiennent. Plus vite ! Aniss tourne trop vite. Le tissu claque un peu. Sarah veut la ronde, elle aussi. Plus vite ! Le tourbillon serre trop. Sa poitrine est coincée. Le sourire de Sarah disparaît. Ses épaules montent. Oh. Tu vois Aniss, Sarah ? Oui, papa. Tes épaules sont hautes, Sarah ? Un peu, maman. L'éclat de rideau tremble, puis tient. Sarah serre les mains trop fort. C'est trop, papa. Papa s'accroupit à la même hauteur. Sarah regarde papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>éclat de rideau</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,80 +1326,63 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis trop_plein; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_ronde_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une bande de soleil rampe sur le plancher.
-narrateur|Le bois est tiède sous les pieds nus.
-narrateur|La maison sent le pain chaud.
-narrateur|Un moulin en papier tourne à la fenêtre.
-narrateur|Il fait un petit bruit doux.
-narrateur|Papa range des livres près du canapé.
-narrateur|Les livres tapent tout bas.
-papa|J'aime ce petit bruit, Victorino.
-papa|Tu as entendu le moulin ?
-enfant-m|Oui, papa. Il tourne.
-narrateur|Le tapis beige est épais.
-narrateur|En ce moment, Victorino joue avec Aniss.
-narrateur|Ils se tiennent par les mains.
-narrateur|Ils tournent au milieu du salon.
-narrateur|Le tapis tourne autour d'eux.
-enfant-m|Plus vite, Aniss !
-narrateur|Aniss tourne plus vite.
-narrateur|Trop vite.
-narrateur|Victorino est gêné.
-narrateur|Aniss le tourne trop fort.
+          <t>narrateur|Le linge tiède bouge devant le jardin.
+narrateur|Ça sent le pain et le soleil.
+enfant-f|Ça sent le pain, papa.
+papa|Tu le sens, le linge, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Un rai passe à travers le tissu.
+narrateur|Le tissu fait un bruit court.
+enfant-f|Il claque, maman.
+maman|Le tissu tient près du bois ?
+enfant-f|Oui, maman.
+narrateur|Près du tissu, un éclat de rideau brille.
+enfant-f|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|La fenêtre tient un bout de jardin pâle.
+enfant-f|Il est clair, papa.
+papa|Le jardin, là-bas ?
+enfant-f|Oui, là-bas.
+narrateur|Aniss tend les mains vers Sarah.
+copain|On tourne, Sarah !
+enfant-f|On tourne, maintenant !
+papa|La ronde, avec Aniss ?
+enfant-f|Oui.
+enfant-f|Tout de suite.
+narrateur|En ce moment, Sarah se penche vers lui.
+narrateur|Leurs mains se tiennent.
+copain|Plus vite !
+narrateur|Aniss tourne trop vite.
+narrateur|Le tissu claque un peu.
+narrateur|Sarah veut la ronde, elle aussi.
+enfant-f|Plus vite !
+narrateur|Le tourbillon serre trop.
 narrateur|Sa poitrine est coincée.
+narrateur|Le sourire de Sarah disparaît.
 narrateur|Ses épaules montent.
-enfant-m|Je n'aime pas.
-enfant-m|C'est trop.
-enfant-m|Stop.
-narrateur|Victorino recule d'un pas.
-narrateur|Il peut s'éloigner.
-narrateur|Il s'éloigne vers le canapé.
-narrateur|Papa est l'adulte près du canapé.
-enfant-m|Papa, c'était trop.
-papa|Tu as dit stop.
-papa|Bravo, Victorino.
-papa|Tu t'es éloigné.
-papa|Tu es venu vers moi.
-papa|Tu veux t'asseoir un peu ?
-enfant-m|Oui, papa.
-narrateur|Victorino pose sa main dans la main de papa.
-narrateur|Il souffle.
-narrateur|Ses épaules descendent.
-papa|Dire stop, c'est permis.
-papa|On s'éloigne.
-papa|On va vers un adulte.
-narrateur|Plus tard, la porte du jardin cliquette.
-narrateur|L'herbe sent le thym.
-narrateur|Un seau jaune attend près des fleurs.
-narrateur|Aniss veut une ronde.
-narrateur|Il prend la main de Victorino.
-narrateur|La ronde commence.
-narrateur|Trop près.
-narrateur|Trop vite encore.
-narrateur|Victorino sent encore sa poitrine coincée.
-narrateur|Il se souvient.
-enfant-m|Stop.
-narrateur|Il s'éloigne.
-narrateur|Il va vers papa, l'adulte.
-enfant-m|Papa, c'est trop encore.
-papa|Tu as repris le geste.
-papa|Bravo.
-papa|Tu as dit stop au jardin aussi.
-papa|Tu t'es éloigné.
-papa|Tu es venu vers un adulte.
-papa|Vers moi.
-narrateur|Victorino reste près de papa.
-narrateur|Ses épaules descendent.
-narrateur|Aniss joue avec le seau jaune.
-narrateur|Le seau tapote l'herbe.</t>
+enfant-f|Oh.
+papa|Tu vois Aniss, Sarah ?
+enfant-f|Oui, papa.
+maman|Tes épaules sont hautes, Sarah ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de rideau tremble, puis tient.
+narrateur|Sarah serre les mains trop fort.
+enfant-f|C'est trop, papa.
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Sarah regarde papa.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>moulin_papier,porte_jardin</t>
+          <t>rideau</t>
         </is>
       </c>
     </row>
@@ -1426,17 +1409,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Victorino. Que dit-il ?</t>
+          <t>C'est trop pour Sarah. Que dit-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Victorino. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;C'est trop pour &lt;emphasis level="moderate"&gt;Sarah&lt;/emphasis&gt;. Que dit-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Sara. Que dit-elle ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;C'est trop pour &lt;emphasis&gt;Sarah&lt;/emphasis&gt;. Que dit-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1461,7 +1444,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Sara dit stop. Puis elle va où ?</t>
+          <t>Sarah dit stop. Puis elle va où ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1499,18 +1482,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1525,34 +1508,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Sarah</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1561,28 +1548,29 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=c_est_trop_que_dit_sarah; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|C'est trop pour Victorino. Que dit-il ?</t>
+          <t>narrateur|C'est trop pour Sarah.
+narrateur|Que dit-elle ?</t>
         </is>
       </c>
     </row>
@@ -1609,17 +1597,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Victorino a dit stop. Il a pu s'éloigner. Il a rejoint papa, l'adulte. Au salon, puis au jardin. Tu as dit le mot juste. Stop. Bravo, Victorino. Tu veux rester près de moi ? Oui. Le thym sent encore. Le seau jaune brille.</t>
+          <t>Sarah veut la ronde, maintenant. Plus vite, Aniss ! Aniss tourne trop, trop près. Le tissu claque contre le bois. Sa poitrine reste coincée. Le sourire ne revient pas. Oh. Sarah refuse de foncer. Stop. Elle recule d'un pas. Les mains se lâchent. Aniss s'arrête net. Ah. Tu restes près de nous, Sarah ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose les mains, puis on reste. D'accord. Sarah reste un moment, les mains ouvertes. Elle souffle. On tourne moins vite ? Moins vite. D'accord. Merci, Sarah. Papa a vu les deux, près du rideau. Le tissu est tiède, sous les doigts. Il est chaud. Sarah glisse la main sur le tissu. Le petit point. Il brille, là ? Oui, là. Sarah pose les mains sur le bois. Elle reste, sans se presser. Tes mains sont au chaud, Sarah ? Un peu, maman. Aniss s'assoit plus droit. Moins vite, oui. Le rideau tient près de la fenêtre ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Victorino a dit stop. Il a pu s'éloigner. Il a rejoint papa, l'adulte. Au salon, puis au jardin. Tu as dit le mot juste. Stop. Bravo, Victorino. Tu veux rester près de moi ? Oui. Le thym sent encore. Le seau jaune brille.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah veut la ronde, maintenant. Plus vite, Aniss ! Aniss tourne trop, trop près. Le tissu claque contre le bois. Sa poitrine reste coincée. Le sourire ne revient pas. Oh. Sarah refuse de foncer. &lt;emphasis level="moderate"&gt;Stop&lt;/emphasis&gt;. Elle recule d'un pas. Les mains se lâchent. Aniss s'arrête net. Ah. Tu restes près de nous, Sarah ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose les mains, puis on reste. D'accord. Sarah reste un moment, les mains ouvertes. Elle souffle. On tourne moins vite ? Moins vite. D'accord. Merci, Sarah. Papa a vu les deux, près du rideau. Le tissu est tiède, sous les doigts. Il est chaud. Sarah glisse la main sur le tissu. Le petit point. Il brille, là ? Oui, là. Sarah pose les mains sur le bois. Elle reste, sans se presser. Tes mains sont au chaud, Sarah ? Un peu, maman. Aniss s'assoit plus droit. Moins vite, oui. Le rideau tient près de la fenêtre ? Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Sara a dit &lt;emphasis&gt;stop&lt;/emphasis&gt;. Elle a pu s'éloigner. Elle rejoint papa, l'adulte. Au salon, puis au jardin. [pause]</t>
+          <t>Sarah veut la ronde, maintenant. Plus vite, Aniss ! Aniss tourne trop, trop près. Le tissu claque contre le bois. Sa poitrine reste coincée. Le sourire ne revient pas. Oh. Sarah refuse de foncer. &lt;emphasis&gt;Stop&lt;/emphasis&gt;. Elle recule d'un pas. Les mains se lâchent. Aniss s'arrête net. Ah. Tu restes près de nous, Sarah ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose les mains, puis on reste. D'accord. Sarah reste un moment, les mains ouvertes. Elle souffle. On tourne moins vite ? Moins vite. D'accord. Merci, Sarah. Papa a vu les deux, près du rideau. Le tissu est tiède, sous les doigts. Il est chaud. Sarah glisse la main sur le tissu. Le petit point. Il brille, là ? Oui, là. Sarah pose les mains sur le bois. Elle reste, sans se presser. Tes mains sont au chaud, Sarah ? Un peu, maman. Aniss s'assoit plus droit. Moins vite, oui. Le rideau tient près de la fenêtre ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1666,7 +1654,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1674,10 +1662,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1700,30 +1688,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>Stop</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1732,10 +1720,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1748,22 +1736,55 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=trop_plein puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_dit_stop_recule; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Victorino a dit stop.
-narrateur|Il a pu s'éloigner.
-narrateur|Il a rejoint papa, l'adulte.
-narrateur|Au salon, puis au jardin.
-papa|Tu as dit le mot juste.
-papa|Stop.
-papa|Bravo, Victorino.
-papa|Tu veux rester près de moi ?
-enfant-m|Oui.
-narrateur|Le thym sent encore.
-narrateur|Le seau jaune brille.</t>
+          <t>narrateur|Sarah veut la ronde, maintenant.
+enfant-f|Plus vite, Aniss !
+narrateur|Aniss tourne trop, trop près.
+narrateur|Le tissu claque contre le bois.
+narrateur|Sa poitrine reste coincée.
+narrateur|Le sourire ne revient pas.
+enfant-f|Oh.
+narrateur|Sarah refuse de foncer.
+enfant-f|Stop.
+narrateur|Elle recule d'un pas.
+narrateur|Les mains se lâchent.
+narrateur|Aniss s'arrête net.
+copain|Ah.
+papa|Tu restes près de nous, Sarah ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Papa, on fait quoi ?
+papa|On pose les mains, puis on reste.
+enfant-f|D'accord.
+narrateur|Sarah reste un moment, les mains ouvertes.
+narrateur|Elle souffle.
+copain|On tourne moins vite ?
+enfant-f|Moins vite.
+copain|D'accord.
+papa|Merci, Sarah.
+narrateur|Papa a vu les deux, près du rideau.
+maman|Le tissu est tiède, sous les doigts.
+enfant-f|Il est chaud.
+narrateur|Sarah glisse la main sur le tissu.
+enfant-f|Le petit point.
+papa|Il brille, là ?
+enfant-f|Oui, là.
+narrateur|Sarah pose les mains sur le bois.
+narrateur|Elle reste, sans se presser.
+maman|Tes mains sont au chaud, Sarah ?
+enfant-f|Un peu, maman.
+narrateur|Aniss s'assoit plus droit.
+enfant-f|Moins vite, oui.
+maman|Le rideau tient près de la fenêtre ?
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>tissu</t>
         </is>
       </c>
     </row>
@@ -1790,17 +1811,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Victorino s'assoit sur le banc du jardin. Le bois du banc est chaud. Papa s'assoit près de lui. On reste un peu ici ? Oui, papa. Tu as bien écouté ton corps. Ta poitrine est plus calme maintenant ? Oui. Plus calme. Un oiseau chante dans le thym. Victorino pose sa main dans la main de papa. Il souffle encore une fois. Le seau jaune est plein de terre. Aniss le montre de loin. Aniss joue tout seul, là-bas. Toi, tu restes ici. C'est bien.</t>
+          <t>Ils restent près de la fenêtre. La porte du jardin s'ouvre. Et dehors, on tourne. Aniss tend les mains. La ronde, maintenant ! Sarah ouvre les bras trop vite. Le tourbillon pousse contre sa poitrine. Sarah avance les pieds, trop vite. Puis elle s'arrête net. Stop. Elle recule d'un pas, vers l'herbe. Personne ne tourne. Elle observe le jardin, un instant. Elle écoute le silence de l'herbe. Au bord du tissu, un éclat de rideau luit. Là, sur le tissu. On tourne moins vite, Aniss ? Aniss ne dit rien, d'abord. Il tient ses mains, sans tourner. Moins vite. Sarah hoche la tête, sans se presser. Aniss souffle, plus lentement. L'herbe est lisse et tiède. Tu l'entends, le jardin ? Oui, papa. La porte est près des fleurs ? Oui, maman. Un panier roule vers le bord. Sarah pose une main dessus. Aniss pose la suivante. Le panier tient, Sarah ? Oui, papa. Un rayon passe sur le rideau. Il allume le tissu.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Victorino s'assoit sur le banc du jardin. Le bois du banc est chaud. Papa s'assoit près de lui. On reste un peu ici ? Oui, papa. Tu as bien écouté ton corps. Ta poitrine est plus calme maintenant ? Oui. Plus calme. Un oiseau chante dans le thym. Victorino pose sa main dans la main de papa. Il souffle encore une fois. Le seau jaune est plein de terre. Aniss le montre de loin. Aniss joue tout seul, là-bas. Toi, tu restes ici. C'est bien.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils restent près de la fenêtre. La porte du jardin s'ouvre. Et dehors, on tourne. Aniss tend les mains. La ronde, maintenant ! Sarah ouvre les bras trop vite. Le tourbillon pousse contre sa poitrine. Sarah avance les pieds, trop vite. Puis elle s'arrête net. Stop. Elle recule d'un pas, vers l'herbe. Personne ne tourne. Elle observe le jardin, un instant. Elle écoute le silence de l'herbe. Au bord du tissu, un &lt;emphasis level="moderate"&gt;éclat de rideau&lt;/emphasis&gt; luit. Là, sur le tissu. On tourne moins vite, Aniss ? Aniss ne dit rien, d'abord. Il tient ses mains, sans tourner. Moins vite. Sarah hoche la tête, sans se presser. Aniss souffle, plus lentement. L'herbe est lisse et tiède. Tu l'entends, le jardin ? Oui, papa. La porte est près des fleurs ? Oui, maman. Un panier roule vers le bord. Sarah pose une main dessus. Aniss pose la suivante. Le panier tient, Sarah ? Oui, papa. Un rayon passe sur le rideau. Il allume le tissu.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Sara reste près du banc. Papa lui parle tout bas. [pause]</t>
+          <t>Ils restent près de la fenêtre. La porte du jardin s'ouvre. Et dehors, on tourne. Aniss tend les mains. La ronde, maintenant ! Sarah ouvre les bras trop vite. Le tourbillon pousse contre sa poitrine. Sarah avance les pieds, trop vite. Puis elle s'arrête net. Stop. Elle recule d'un pas, vers l'herbe. Personne ne tourne. Elle observe le jardin, un instant. Elle écoute le silence de l'herbe. Au bord du tissu, un &lt;emphasis&gt;éclat de rideau&lt;/emphasis&gt; luit. Là, sur le tissu. On tourne moins vite, Aniss ? Aniss ne dit rien, d'abord. Il tient ses mains, sans tourner. Moins vite. Sarah hoche la tête, sans se presser. Aniss souffle, plus lentement. L'herbe est lisse et tiède. Tu l'entends, le jardin ? Oui, papa. La porte est près des fleurs ? Oui, maman. Un panier roule vers le bord. Sarah pose une main dessus. Aniss pose la suivante. Le panier tient, Sarah ? Oui, papa. Un rayon passe sur le rideau. Il allume le tissu. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1847,7 +1868,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1855,10 +1876,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1879,28 +1900,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de rideau</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1909,10 +1934,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1923,30 +1948,52 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=jardin_trop_vite_elle_dit_stop; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Victorino s'assoit sur le banc du jardin.
-narrateur|Le bois du banc est chaud.
-narrateur|Papa s'assoit près de lui.
-papa|On reste un peu ici ?
-enfant-m|Oui, papa.
-papa|Tu as bien écouté ton corps.
-papa|Ta poitrine est plus calme maintenant ?
-enfant-m|Oui. Plus calme.
-narrateur|Un oiseau chante dans le thym.
-narrateur|Victorino pose sa main dans la main de papa.
-narrateur|Il souffle encore une fois.
-narrateur|Le seau jaune est plein de terre.
-narrateur|Aniss le montre de loin.
-papa|Aniss joue tout seul, là-bas.
-papa|Toi, tu restes ici.
-papa|C'est bien.</t>
+          <t>narrateur|Ils restent près de la fenêtre.
+narrateur|La porte du jardin s'ouvre.
+copain|Et dehors, on tourne.
+narrateur|Aniss tend les mains.
+enfant-f|La ronde, maintenant !
+narrateur|Sarah ouvre les bras trop vite.
+narrateur|Le tourbillon pousse contre sa poitrine.
+narrateur|Sarah avance les pieds, trop vite.
+narrateur|Puis elle s'arrête net.
+enfant-f|Stop.
+narrateur|Elle recule d'un pas, vers l'herbe.
+narrateur|Personne ne tourne.
+narrateur|Elle observe le jardin, un instant.
+narrateur|Elle écoute le silence de l'herbe.
+narrateur|Au bord du tissu, un éclat de rideau luit.
+enfant-f|Là, sur le tissu.
+enfant-f|On tourne moins vite, Aniss ?
+narrateur|Aniss ne dit rien, d'abord.
+narrateur|Il tient ses mains, sans tourner.
+copain|Moins vite.
+narrateur|Sarah hoche la tête, sans se presser.
+narrateur|Aniss souffle, plus lentement.
+narrateur|L'herbe est lisse et tiède.
+papa|Tu l'entends, le jardin ?
+enfant-f|Oui, papa.
+maman|La porte est près des fleurs ?
+enfant-f|Oui, maman.
+narrateur|Un panier roule vers le bord.
+narrateur|Sarah pose une main dessus.
+narrateur|Aniss pose la suivante.
+papa|Le panier tient, Sarah ?
+enfant-f|Oui, papa.
+maman|Un rayon passe sur le rideau.
+enfant-f|Il allume le tissu.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>oiseau</t>
+          <t>porte_jardin</t>
         </is>
       </c>
     </row>
@@ -1973,17 +2020,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je me suis éloigné. Je suis allé vers papa. Bravo. Au salon, et au jardin.</t>
+          <t>Ils restent près de la porte. La ronde a eu son tour, Sarah ? Oui, maman. Tu souffles un peu ? Oui, papa. Sarah souffle, un filet d'air. Le tissu sent bon. Tu le sens, le linge ? Oui, maman. Le rideau reste un peu, à plat. Il a tenu, sur le bois. Le jardin est chaud, sous les mains. L'herbe fait une petite ombre. On y revient, après. Un éclat de rideau tient sur le tissu.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je me suis éloigné. Je suis allé vers papa. Bravo. Au salon, et au jardin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la porte. La ronde a eu son tour, Sarah ? Oui, maman. Tu souffles un peu ? Oui, papa. Sarah souffle, un filet d'air. Le tissu sent bon. Tu le sens, le linge ? Oui, maman. Le rideau reste un peu, à plat. Il a tenu, sur le bois. Le jardin est chaud, sous les mains. L'herbe fait une petite ombre. On y revient, après. Un &lt;emphasis level="moderate"&gt;éclat de rideau&lt;/emphasis&gt; tient sur le tissu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la porte. La ronde a eu son tour, Sarah ? Oui, maman. Tu souffles un peu ? Oui, papa. Sarah souffle, un filet d'air. Le tissu sent bon. Tu le sens, le linge ? Oui, maman. Le rideau reste un peu, à plat. Il a tenu, sur le bois. Le jardin est chaud, sous les mains. L'herbe fait une petite ombre. On y revient, après. Un &lt;emphasis&gt;éclat de rideau&lt;/emphasis&gt; tient sur le tissu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2030,18 +2077,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2050,12 +2097,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2064,17 +2111,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de rideau</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2083,11 +2134,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2096,28 +2147,42 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_tissu; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai dit stop.
-enfant-m|Je me suis éloigné.
-enfant-m|Je suis allé vers papa.
-papa|Bravo.
-papa|Au salon, et au jardin.</t>
+          <t>narrateur|Ils restent près de la porte.
+maman|La ronde a eu son tour, Sarah ?
+enfant-f|Oui, maman.
+papa|Tu souffles un peu ?
+enfant-f|Oui, papa.
+narrateur|Sarah souffle, un filet d'air.
+enfant-f|Le tissu sent bon.
+maman|Tu le sens, le linge ?
+enfant-f|Oui, maman.
+papa|Le rideau reste un peu, à plat.
+enfant-f|Il a tenu, sur le bois.
+narrateur|Le jardin est chaud, sous les mains.
+narrateur|L'herbe fait une petite ombre.
+enfant-f|On y revient, après.
+narrateur|Un éclat de rideau tient sur le tissu.</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2195,6 +2260,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>